<commit_message>
fix: corrected confusion matrix metrics (TP/FP/FN/TN) to standard ML convention and enhanced downstream policy inconsistency detection with unresolved endpoint handling
Updated metrics computation to properly classify inconsistency detection outcomes using standard ML definitions where TP=correctly flags inconsistency, FP=false alarm, FN=misses real inconsistency, TN=correctly reports consistent. Fixed Excel formulas for TPR/FPR/FNR calculations and corrected parameter specification rate denominator.
</commit_message>
<xml_diff>
--- a/yas/first-injection/output/metrics.xlsx
+++ b/yas/first-injection/output/metrics.xlsx
@@ -623,7 +623,7 @@
         <v>2</v>
       </c>
       <c r="P6">
-        <f>IF(O6&gt;0,O6/N6,0)</f>
+        <f>IF(O6&gt;0,N6/O6,0)</f>
         <v/>
       </c>
     </row>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="P7">
-        <f>IF(O7&gt;0,O7/N7,0)</f>
+        <f>IF(O7&gt;0,N7/O7,0)</f>
         <v/>
       </c>
     </row>
@@ -737,7 +737,7 @@
         <v>0</v>
       </c>
       <c r="P8">
-        <f>IF(O8&gt;0,O8/N8,0)</f>
+        <f>IF(O8&gt;0,N8/O8,0)</f>
         <v/>
       </c>
     </row>
@@ -768,7 +768,7 @@
         <v/>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I9" t="n">
         <v>6</v>
@@ -794,7 +794,7 @@
         <v>2</v>
       </c>
       <c r="P9">
-        <f>IF(O9&gt;0,O9/N9,0)</f>
+        <f>IF(O9&gt;0,N9/O9,0)</f>
         <v/>
       </c>
     </row>
@@ -825,7 +825,7 @@
         <v/>
       </c>
       <c r="H10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
         <v>3</v>
@@ -848,10 +848,10 @@
         <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P10">
-        <f>IF(O10&gt;0,O10/N10,0)</f>
+        <f>IF(O10&gt;0,N10/O10,0)</f>
         <v/>
       </c>
     </row>
@@ -885,7 +885,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J11">
         <f>IF(I11&gt;0,(H11/I11)*100,0)</f>
@@ -908,7 +908,7 @@
         <v>0</v>
       </c>
       <c r="P11">
-        <f>IF(O11&gt;0,O11/N11,0)</f>
+        <f>IF(O11&gt;0,N11/O11,0)</f>
         <v/>
       </c>
     </row>
@@ -939,7 +939,7 @@
         <v/>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" t="n">
         <v>4</v>
@@ -965,18 +965,18 @@
         <v>2</v>
       </c>
       <c r="P12">
-        <f>IF(O12&gt;0,O12/N12,0)</f>
+        <f>IF(O12&gt;0,N12/O12,0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DELETE /ApiConstant.WAREHOUSE_URL/{?}</t>
+          <t>DELETE /backoffice/warehouses/{?}</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
         <v>4</v>
@@ -986,7 +986,7 @@
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>1</v>
@@ -996,10 +996,10 @@
         <v/>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J13">
         <f>IF(I13&gt;0,(H13/I13)*100,0)</f>
@@ -1009,20 +1009,20 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13">
         <f>IF(L13+K13&gt;0,K13/(K13+L13),0)</f>
         <v/>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P13">
-        <f>IF(O13&gt;0,O13/N13,0)</f>
+        <f>IF(O13&gt;0,N13/O13,0)</f>
         <v/>
       </c>
     </row>
@@ -1079,18 +1079,18 @@
         <v>2</v>
       </c>
       <c r="P14">
-        <f>IF(O14&gt;0,O14/N14,0)</f>
+        <f>IF(O14&gt;0,N14/O14,0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PUT /Constants.ApiConstant.STATE_OR_PROVINCES_URL/{?}</t>
+          <t>PUT /backoffice/state-or-provinces/{?}</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
         <v>4</v>
@@ -1100,7 +1100,7 @@
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
@@ -1120,7 +1120,7 @@
         <v/>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1130,13 +1130,13 @@
         <v/>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P15">
-        <f>IF(O15&gt;0,O15/N15,0)</f>
+        <f>IF(O15&gt;0,N15/O15,0)</f>
         <v/>
       </c>
     </row>
@@ -1165,17 +1165,17 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>True Negative Rate</t>
+          <t>True Positive Rate (TPR)</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>False Negative Rate</t>
+          <t>False Positive Rate (FPR)</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>False Positive Rate</t>
+          <t>False Negative Rate (FNR)</t>
         </is>
       </c>
       <c r="T20" s="2" t="inlineStr">
@@ -1247,47 +1247,47 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Cases that correctly captures inconsistency (TN)</t>
+          <t>True Positives: correctly flags inconsistency (TP)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Cases that missed inconsistency (FP)</t>
+          <t>False Negatives: misses real inconsistency (FN)</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>TNR</t>
+          <t>TPR = TP/(TP+FN)</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Cases that incorrectly captures inconsistencies (FN)</t>
+          <t>False Positives: false alarm (FP)</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cases that tests consistency (TP) </t>
+          <t>True Negatives: correctly reports consistent (TN)</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>FNR</t>
+          <t>FPR = FP/(FP+TN)</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>Cases that missed inconsistency (FP)</t>
+          <t>False Positives: false alarm (FP)</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>Cases that correctly captures inconsistency (TN)</t>
+          <t>True Negatives: correctly reports consistent (TN)</t>
         </is>
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>FPR</t>
+          <t>FNR = FN/(FN+TP)</t>
         </is>
       </c>
       <c r="T21" s="2" t="inlineStr">
@@ -1333,10 +1333,10 @@
         <v/>
       </c>
       <c r="H22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J22">
         <f>IF(I22&gt;0,(H22/I22)*100,0)</f>
@@ -1377,7 +1377,7 @@
         <v/>
       </c>
       <c r="U22">
-        <f>IF(K22+Q22&gt;0,K22/(K22+Q22),0)</f>
+        <f>IF(K22+L22&gt;0,K22/(K22+L22),0)</f>
         <v/>
       </c>
       <c r="V22">
@@ -1412,10 +1412,10 @@
         <v/>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J23">
         <f>IF(I23&gt;0,(H23/I23)*100,0)</f>
@@ -1456,7 +1456,7 @@
         <v/>
       </c>
       <c r="U23">
-        <f>IF(K23+Q23&gt;0,K23/(K23+Q23),0)</f>
+        <f>IF(K23+L23&gt;0,K23/(K23+L23),0)</f>
         <v/>
       </c>
       <c r="V23">
@@ -1491,10 +1491,10 @@
         <v/>
       </c>
       <c r="H24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J24">
         <f>IF(I24&gt;0,(H24/I24)*100,0)</f>
@@ -1535,7 +1535,7 @@
         <v/>
       </c>
       <c r="U24">
-        <f>IF(K24+Q24&gt;0,K24/(K24+Q24),0)</f>
+        <f>IF(K24+L24&gt;0,K24/(K24+L24),0)</f>
         <v/>
       </c>
       <c r="V24">
@@ -1550,7 +1550,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
         <v>4</v>
@@ -1570,10 +1570,10 @@
         <v/>
       </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J25">
         <f>IF(I25&gt;0,(H25/I25)*100,0)</f>
@@ -1614,7 +1614,7 @@
         <v/>
       </c>
       <c r="U25">
-        <f>IF(K25+Q25&gt;0,K25/(K25+Q25),0)</f>
+        <f>IF(K25+L25&gt;0,K25/(K25+L25),0)</f>
         <v/>
       </c>
       <c r="V25">
@@ -1649,17 +1649,17 @@
         <v/>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J26">
         <f>IF(I26&gt;0,(H26/I26)*100,0)</f>
         <v/>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -1669,7 +1669,7 @@
         <v/>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
@@ -1682,7 +1682,7 @@
         <v>0</v>
       </c>
       <c r="R26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S26">
         <f>IF(Q26+R26&gt;0,Q26/(Q26+R26),0)</f>
@@ -1693,7 +1693,7 @@
         <v/>
       </c>
       <c r="U26">
-        <f>IF(K26+Q26&gt;0,K26/(K26+Q26),0)</f>
+        <f>IF(K26+L26&gt;0,K26/(K26+L26),0)</f>
         <v/>
       </c>
       <c r="V26">
@@ -1718,7 +1718,7 @@
         <v/>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>4</v>
@@ -1728,10 +1728,10 @@
         <v/>
       </c>
       <c r="H27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J27">
         <f>IF(I27&gt;0,(H27/I27)*100,0)</f>
@@ -1741,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27">
         <f>IF(K27+L27&gt;0,K27/(K27+L27),0)</f>
@@ -1751,14 +1751,14 @@
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P27">
         <f>IF(N27+O27&gt;0,N27/(N27+O27),0)</f>
         <v/>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -1772,7 +1772,7 @@
         <v/>
       </c>
       <c r="U27">
-        <f>IF(K27+Q27&gt;0,K27/(K27+Q27),0)</f>
+        <f>IF(K27+L27&gt;0,K27/(K27+L27),0)</f>
         <v/>
       </c>
       <c r="V27">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C28" t="n">
         <v>4</v>
@@ -1807,10 +1807,10 @@
         <v/>
       </c>
       <c r="H28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <f>IF(I28&gt;0,(H28/I28)*100,0)</f>
@@ -1851,7 +1851,7 @@
         <v/>
       </c>
       <c r="U28">
-        <f>IF(K28+Q28&gt;0,K28/(K28+Q28),0)</f>
+        <f>IF(K28+L28&gt;0,K28/(K28+L28),0)</f>
         <v/>
       </c>
       <c r="V28">
@@ -1862,34 +1862,34 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DELETE /ApiConstant.WAREHOUSE_URL/{?}</t>
+          <t>DELETE /backoffice/warehouses/{?}</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D29">
         <f>IF(C29&gt;0,(B29/C29)*100,0)</f>
         <v/>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G29">
         <f>(E29/F29)*100</f>
         <v/>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29">
         <f>IF(I29&gt;0,(H29/I29)*100,0)</f>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29">
         <f>IF(K29+L29&gt;0,K29/(K29+L29),0)</f>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -1930,7 +1930,7 @@
         <v/>
       </c>
       <c r="U29">
-        <f>IF(K29+Q29&gt;0,K29/(K29+Q29),0)</f>
+        <f>IF(K29+L29&gt;0,K29/(K29+L29),0)</f>
         <v/>
       </c>
       <c r="V29">
@@ -1965,10 +1965,10 @@
         <v/>
       </c>
       <c r="H30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J30">
         <f>IF(I30&gt;0,(H30/I30)*100,0)</f>
@@ -2009,7 +2009,7 @@
         <v/>
       </c>
       <c r="U30">
-        <f>IF(K30+Q30&gt;0,K30/(K30+Q30),0)</f>
+        <f>IF(K30+L30&gt;0,K30/(K30+L30),0)</f>
         <v/>
       </c>
       <c r="V30">
@@ -2020,34 +2020,34 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PUT /Constants.ApiConstant.STATE_OR_PROVINCES_URL/{?}</t>
+          <t>PUT /backoffice/state-or-provinces/{?}</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D31">
         <f>IF(C31&gt;0,(B31/C31)*100,0)</f>
         <v/>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G31">
         <f>(E31/F31)*100</f>
         <v/>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31">
         <f>IF(I31&gt;0,(H31/I31)*100,0)</f>
@@ -2088,7 +2088,7 @@
         <v/>
       </c>
       <c r="U31">
-        <f>IF(K31+Q31&gt;0,K31/(K31+Q31),0)</f>
+        <f>IF(K31+L31&gt;0,K31/(K31+L31),0)</f>
         <v/>
       </c>
       <c r="V31">

</xml_diff>